<commit_message>
Deploy updated output folder
</commit_message>
<xml_diff>
--- a/CodeSystem-nigeria-facility-type.xlsx
+++ b/CodeSystem-nigeria-facility-type.xlsx
@@ -24,7 +24,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>https://dhin.org/2025Connectathon/CodeSystem/nigeria-facility-type</t>
+    <t>https://www.dhin-hie.org/IGs/CodeSystem/nigeria-facility-type</t>
   </si>
   <si>
     <t>Version</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-08-02T14:19:18+01:00</t>
+    <t>2025-09-10T08:54:29+01:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>